<commit_message>
Integrate real resource data and capacity dashboard
</commit_message>
<xml_diff>
--- a/docs/ai_monitoring_metric_dictionary.xlsx
+++ b/docs/ai_monitoring_metric_dictionary.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readme" sheetId="1" r:id="Rc7a24d2d44b64aae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrics" sheetId="2" r:id="R28dadb493f724a93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fields" sheetId="3" r:id="R220d5405ad4d4db1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alert Rules" sheetId="4" r:id="R36b8fd2424b447e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimensions" sheetId="5" r:id="Rd92142a1d96b4c7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config Values" sheetId="6" r:id="R1cd974703435437b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version History" sheetId="7" r:id="R4d3bdaf686464066"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composite Rules" sheetId="8" r:id="R5afed994f0484628"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Conditions" sheetId="9" r:id="Rbd6101fbb69b474e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fusion Strategies" sheetId="10" r:id="R3346e5b6e54e4d17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fusion Grading" sheetId="11" r:id="Rd0ea0223f1f74a4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Probes" sheetId="12" r:id="R2889d2d95ae34a49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Probe Assertions" sheetId="13" r:id="R13da75c3d6784524"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Severity Policy" sheetId="14" r:id="Rd400e8f0ab114c4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Policy" sheetId="15" r:id="Ra7ab83e2fa31417c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Tasks" sheetId="16" r:id="R8441a931cf344b52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagnosis Policy" sheetId="17" r:id="Rca77a90a0b504f3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Policy" sheetId="18" r:id="R639808bb4a7040ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readme" sheetId="1" r:id="R892211a0674b4423"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrics" sheetId="2" r:id="R1fda3da71e57475d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fields" sheetId="3" r:id="R6859e0b2ae4f47e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alert Rules" sheetId="4" r:id="R3230084c58284f35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimensions" sheetId="5" r:id="R432b2532af8746d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config Values" sheetId="6" r:id="R0b51b30019974f2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version History" sheetId="7" r:id="Rbc8fccf5d4244a16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composite Rules" sheetId="8" r:id="R71d575617ee741ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Conditions" sheetId="9" r:id="Rfaa1f667fe774504"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fusion Strategies" sheetId="10" r:id="R5afe9000162940c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fusion Grading" sheetId="11" r:id="R88ee130b4f9c4cd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Probes" sheetId="12" r:id="R130c2e01abf04a81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Probe Assertions" sheetId="13" r:id="R389ceceba8d24b25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Severity Policy" sheetId="14" r:id="R26c4a0a89c26481c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Policy" sheetId="15" r:id="R687390f845ae4252"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Tasks" sheetId="16" r:id="R81697d1596404160"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagnosis Policy" sheetId="17" r:id="R8608806e173e4620"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Policy" sheetId="18" r:id="R8647e6784af446c4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2161,7 +2161,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70f1f36a639541dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16d5c59dc2564660"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2358,7 +2358,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24708a25056c446c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4da13a4139045f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2460,19 +2460,19 @@
         <x:v>PROBE-001</x:v>
       </x:c>
       <x:c r="B2" s="88" t="str">
-        <x:v>OPENAI_PING_EAST</x:v>
+        <x:v>MINIMAX_PING_EAST</x:v>
       </x:c>
       <x:c r="C2" s="88" t="str">
-        <x:v>OpenAI基础可用性</x:v>
+        <x:v>MiniMax基础可用性</x:v>
       </x:c>
       <x:c r="D2" s="88" t="str">
         <x:v>availability</x:v>
       </x:c>
       <x:c r="E2" s="88" t="str">
-        <x:v>OpenAI</x:v>
+        <x:v>MiniMax</x:v>
       </x:c>
       <x:c r="F2" s="88" t="str">
-        <x:v>gpt-4.1-mini</x:v>
+        <x:v>Minimax-M2.5</x:v>
       </x:c>
       <x:c r="G2" s="88" t="str">
         <x:v>cn-east</x:v>
@@ -2493,7 +2493,7 @@
         <x:v>1500</x:v>
       </x:c>
       <x:c r="M2" s="88" t="n">
-        <x:v>3000</x:v>
+        <x:v>5000</x:v>
       </x:c>
       <x:c r="N2" s="88" t="n">
         <x:v>8</x:v>
@@ -2502,7 +2502,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="P2" s="88" t="str">
-        <x:v>PROBE_OPENAI_KEY</x:v>
+        <x:v>PROBE_MINIMAX_KEY</x:v>
       </x:c>
       <x:c r="Q2" s="88" t="str">
         <x:v>critical</x:v>
@@ -2517,7 +2517,7 @@
         <x:v>0.4.0</x:v>
       </x:c>
       <x:c r="U2" s="88" t="str">
-        <x:v>确认OpenAI东区基础调用和固定内容返回</x:v>
+        <x:v>确认MiniMax东区基础调用和固定内容返回</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="50" customHeight="1">
@@ -2528,16 +2528,16 @@
         <x:v>QWEN_PING_EAST</x:v>
       </x:c>
       <x:c r="C3" s="88" t="str">
-        <x:v>通义基础可用性</x:v>
+        <x:v>Qwen基础可用性</x:v>
       </x:c>
       <x:c r="D3" s="88" t="str">
         <x:v>availability</x:v>
       </x:c>
       <x:c r="E3" s="88" t="str">
-        <x:v>Alibaba Cloud</x:v>
+        <x:v>Qwen</x:v>
       </x:c>
       <x:c r="F3" s="88" t="str">
-        <x:v>qwen-plus</x:v>
+        <x:v>Qwen3.6-35B-A3B</x:v>
       </x:c>
       <x:c r="G3" s="88" t="str">
         <x:v>cn-east</x:v>
@@ -2558,7 +2558,7 @@
         <x:v>1500</x:v>
       </x:c>
       <x:c r="M3" s="88" t="n">
-        <x:v>3000</x:v>
+        <x:v>5000</x:v>
       </x:c>
       <x:c r="N3" s="88" t="n">
         <x:v>8</x:v>
@@ -2582,7 +2582,7 @@
         <x:v>0.4.0</x:v>
       </x:c>
       <x:c r="U3" s="88" t="str">
-        <x:v>确认通义东区基础调用和固定内容返回</x:v>
+        <x:v>确认Qwen东区基础调用和固定内容返回</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="50" customHeight="1">
@@ -2602,7 +2602,7 @@
         <x:v>DeepSeek</x:v>
       </x:c>
       <x:c r="F4" s="88" t="str">
-        <x:v>deepseek-chat</x:v>
+        <x:v>DeepSeek-V4</x:v>
       </x:c>
       <x:c r="G4" s="88" t="str">
         <x:v>cn-east</x:v>
@@ -2620,10 +2620,10 @@
         <x:v>5000</x:v>
       </x:c>
       <x:c r="L4" s="88" t="n">
-        <x:v>1500</x:v>
+        <x:v>9000</x:v>
       </x:c>
       <x:c r="M4" s="88" t="n">
-        <x:v>3000</x:v>
+        <x:v>15000</x:v>
       </x:c>
       <x:c r="N4" s="88" t="n">
         <x:v>8</x:v>
@@ -2655,19 +2655,19 @@
         <x:v>PROBE-004</x:v>
       </x:c>
       <x:c r="B5" s="88" t="str">
-        <x:v>OPENAI_JSON_NORTH</x:v>
+        <x:v>MINIMAX_JSON_NORTH</x:v>
       </x:c>
       <x:c r="C5" s="88" t="str">
-        <x:v>OpenAI JSON能力</x:v>
+        <x:v>MiniMax JSON能力</x:v>
       </x:c>
       <x:c r="D5" s="88" t="str">
         <x:v>json_schema</x:v>
       </x:c>
       <x:c r="E5" s="88" t="str">
-        <x:v>OpenAI</x:v>
+        <x:v>MiniMax</x:v>
       </x:c>
       <x:c r="F5" s="88" t="str">
-        <x:v>gpt-4.1-mini</x:v>
+        <x:v>Minimax-M2.5</x:v>
       </x:c>
       <x:c r="G5" s="88" t="str">
         <x:v>cn-north</x:v>
@@ -2688,7 +2688,7 @@
         <x:v>2200</x:v>
       </x:c>
       <x:c r="M5" s="88" t="n">
-        <x:v>5000</x:v>
+        <x:v>6000</x:v>
       </x:c>
       <x:c r="N5" s="88" t="n">
         <x:v>24</x:v>
@@ -2697,7 +2697,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="P5" s="88" t="str">
-        <x:v>PROBE_OPENAI_KEY</x:v>
+        <x:v>PROBE_MINIMAX_KEY</x:v>
       </x:c>
       <x:c r="Q5" s="88" t="str">
         <x:v>warning</x:v>
@@ -2723,16 +2723,16 @@
         <x:v>QWEN_STREAM_SOUTH</x:v>
       </x:c>
       <x:c r="C6" s="88" t="str">
-        <x:v>通义流式首Token</x:v>
+        <x:v>Qwen流式首Token</x:v>
       </x:c>
       <x:c r="D6" s="88" t="str">
         <x:v>stream_ttft</x:v>
       </x:c>
       <x:c r="E6" s="88" t="str">
-        <x:v>Alibaba Cloud</x:v>
+        <x:v>Qwen</x:v>
       </x:c>
       <x:c r="F6" s="88" t="str">
-        <x:v>qwen-plus</x:v>
+        <x:v>Qwen3.6-35B-A3B</x:v>
       </x:c>
       <x:c r="G6" s="88" t="str">
         <x:v>cn-south</x:v>
@@ -2797,7 +2797,7 @@
         <x:v>DeepSeek</x:v>
       </x:c>
       <x:c r="F7" s="10" t="str">
-        <x:v>deepseek-chat</x:v>
+        <x:v>DeepSeek-V4</x:v>
       </x:c>
       <x:c r="G7" s="10" t="str">
         <x:v>cn-north</x:v>
@@ -2815,10 +2815,10 @@
         <x:v>9000</x:v>
       </x:c>
       <x:c r="L7" s="10" t="n">
-        <x:v>2500</x:v>
+        <x:v>10000</x:v>
       </x:c>
       <x:c r="M7" s="10" t="n">
-        <x:v>7000</x:v>
+        <x:v>18000</x:v>
       </x:c>
       <x:c r="N7" s="10" t="n">
         <x:v>48</x:v>
@@ -2866,7 +2866,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3798d4a241b94702"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2a550081fef4907"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3217,7 +3217,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree54774d5b614e20"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6e962e00dd14124"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3412,7 +3412,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92964546f8ee4454"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ee5600703d24b07"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5154,7 +5154,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re892d983c0004a40"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1278df2fc31846a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5480,7 +5480,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac91050be4a34370"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd02e685b208640f6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5825,7 +5825,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R692a40f9f706421d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce68f42da8ca4e02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6528,7 +6528,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ab7ce74f1ff4870"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf38653235ae4eea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9396,7 +9396,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0c317888189407d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09a266a2a19a4fd2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9740,7 +9740,7 @@
         <x:v>no</x:v>
       </x:c>
       <x:c r="G7" s="9" t="str">
-        <x:v>gpt-4.1-mini</x:v>
+        <x:v>DeepSeek-V4</x:v>
       </x:c>
       <x:c r="H7" s="9" t="str">
         <x:v>实际处理请求的模型标识</x:v>
@@ -9789,7 +9789,7 @@
         <x:v>no</x:v>
       </x:c>
       <x:c r="G8" s="9" t="str">
-        <x:v>OpenAI</x:v>
+        <x:v>DeepSeek</x:v>
       </x:c>
       <x:c r="H8" s="9" t="str">
         <x:v>模型服务提供方</x:v>
@@ -14671,7 +14671,7 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G104" t="str">
-        <x:v>deepseek-chat</x:v>
+        <x:v>Qwen3.6-35B-A3B</x:v>
       </x:c>
       <x:c r="H104" t="str">
         <x:v>满足跨供应商和健康约束的替代模型</x:v>
@@ -14977,7 +14977,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R452e15d125eb4f88"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R626d25ecabf1493c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15352,7 +15352,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7837c31099f34299"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5262b3b7c2d941e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15778,7 +15778,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd710ba412fe64665"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f2cda8f6e264043"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16070,7 +16070,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98ddb19b8899460b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4525c26d40ea4740"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16684,7 +16684,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c4dfe998b394e93"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bdb237312584556"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17248,7 +17248,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf735e95d23b841e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3611b1a57f5c49ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17765,7 +17765,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bed0c1ef2174b5e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8804abdb906c4c81"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Redesign health performance and cost dashboards
</commit_message>
<xml_diff>
--- a/docs/ai_monitoring_metric_dictionary.xlsx
+++ b/docs/ai_monitoring_metric_dictionary.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readme" sheetId="1" r:id="R892211a0674b4423"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrics" sheetId="2" r:id="R1fda3da71e57475d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fields" sheetId="3" r:id="R6859e0b2ae4f47e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alert Rules" sheetId="4" r:id="R3230084c58284f35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimensions" sheetId="5" r:id="R432b2532af8746d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config Values" sheetId="6" r:id="R0b51b30019974f2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version History" sheetId="7" r:id="Rbc8fccf5d4244a16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composite Rules" sheetId="8" r:id="R71d575617ee741ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Conditions" sheetId="9" r:id="Rfaa1f667fe774504"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fusion Strategies" sheetId="10" r:id="R5afe9000162940c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fusion Grading" sheetId="11" r:id="R88ee130b4f9c4cd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Probes" sheetId="12" r:id="R130c2e01abf04a81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Probe Assertions" sheetId="13" r:id="R389ceceba8d24b25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Severity Policy" sheetId="14" r:id="R26c4a0a89c26481c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Policy" sheetId="15" r:id="R687390f845ae4252"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Tasks" sheetId="16" r:id="R81697d1596404160"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagnosis Policy" sheetId="17" r:id="R8608806e173e4620"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Policy" sheetId="18" r:id="R8647e6784af446c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readme" sheetId="1" r:id="R83b3e0835b2740e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrics" sheetId="2" r:id="Rd7a71123dde44659"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fields" sheetId="3" r:id="Ra62d25f34d9b48ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alert Rules" sheetId="4" r:id="R42ebbcbcce7d46ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimensions" sheetId="5" r:id="Re474d66468264821"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config Values" sheetId="6" r:id="R81566ca83c334479"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version History" sheetId="7" r:id="Re368677e26d341f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composite Rules" sheetId="8" r:id="Rb4efe5d3c1194968"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Conditions" sheetId="9" r:id="R2e0bd43fad2246c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fusion Strategies" sheetId="10" r:id="R58ac61144a89462c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fusion Grading" sheetId="11" r:id="R52c587be9846496b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Probes" sheetId="12" r:id="R05256f45d8ce4a44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Probe Assertions" sheetId="13" r:id="R45946a05cf4e4d40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Severity Policy" sheetId="14" r:id="Rda913d51cdd340e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Policy" sheetId="15" r:id="R6e6268d4fb4645a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Tasks" sheetId="16" r:id="R08c8c0c628d746d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagnosis Policy" sheetId="17" r:id="Rb6009eba43d547fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Policy" sheetId="18" r:id="Rf0db931b35c34f14"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1700,7 +1700,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="28" t="str">
-        <x:v>Version 0.10.0 | Added model health risk recognition and diagnostic evidence center</x:v>
+        <x:v>Version 0.11.0 | Removed duplicate stability weighting from model health score</x:v>
       </x:c>
       <x:c r="B3" s="28"/>
       <x:c r="C3" s="28"/>
@@ -2161,7 +2161,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16d5c59dc2564660"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R144b083b98524f02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2358,7 +2358,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4da13a4139045f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fa6814d83a142ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2866,7 +2866,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2a550081fef4907"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb51ef5fe4b16479f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3217,7 +3217,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6e962e00dd14124"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78b9a933238d4227"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3412,7 +3412,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ee5600703d24b07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc7b162c88cd4168"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4015,7 +4015,7 @@
         <x:v>active</x:v>
       </x:c>
       <x:c r="N15" s="149" t="str">
-        <x:v>0.6.0</x:v>
+        <x:v>0.11.0</x:v>
       </x:c>
       <x:c r="O15" s="149" t="str">
         <x:v>健康指数成功率权重</x:v>
@@ -4038,7 +4038,7 @@
         <x:v>passthrough</x:v>
       </x:c>
       <x:c r="F16" s="150" t="n">
-        <x:v>0.25</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="G16" s="151"/>
       <x:c r="H16" s="151"/>
@@ -4052,10 +4052,10 @@
         <x:v>active</x:v>
       </x:c>
       <x:c r="N16" s="149" t="str">
-        <x:v>0.6.0</x:v>
+        <x:v>0.11.0</x:v>
       </x:c>
       <x:c r="O16" s="149" t="str">
-        <x:v>健康指数性能权重</x:v>
+        <x:v>健康指数性能权重；性能已包含稳定性</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="32" customHeight="1">
@@ -4086,13 +4086,13 @@
         <x:v>score</x:v>
       </x:c>
       <x:c r="M17" s="149" t="str">
-        <x:v>active</x:v>
+        <x:v>inactive</x:v>
       </x:c>
       <x:c r="N17" s="149" t="str">
-        <x:v>0.6.0</x:v>
+        <x:v>0.11.0</x:v>
       </x:c>
       <x:c r="O17" s="149" t="str">
-        <x:v>健康指数稳定性权重</x:v>
+        <x:v>已停用：稳定性已包含在performance_score中，避免重复加权</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="32" customHeight="1">
@@ -4126,7 +4126,7 @@
         <x:v>active</x:v>
       </x:c>
       <x:c r="N18" s="149" t="str">
-        <x:v>0.6.0</x:v>
+        <x:v>0.11.0</x:v>
       </x:c>
       <x:c r="O18" s="149" t="str">
         <x:v>健康指数成本效率权重</x:v>
@@ -5154,7 +5154,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1278df2fc31846a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f569c11fa2f46a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5480,7 +5480,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd02e685b208640f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5313b656fb224b9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5825,7 +5825,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce68f42da8ca4e02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4e148933d234aea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6528,7 +6528,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf38653235ae4eea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd51da43ba80945d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8597,10 +8597,10 @@
         <x:v>operations</x:v>
       </x:c>
       <x:c r="E32" t="str">
-        <x:v>综合成功率、性能、稳定性和成本效率的模型健康得分</x:v>
+        <x:v>综合成功率、性能（已含稳定性）和成本效率的模型健康得分</x:v>
       </x:c>
       <x:c r="F32" t="str">
-        <x:v>0.35 * success_score + 0.25 * performance_score + 0.25 * stability_score + 0.15 * cost_efficiency_score</x:v>
+        <x:v>0.35 * success_score + 0.50 * performance_score + 0.15 * cost_efficiency_score</x:v>
       </x:c>
       <x:c r="G32" t="str">
         <x:v>score</x:v>
@@ -8618,7 +8618,7 @@
         <x:v>model_operating_scores</x:v>
       </x:c>
       <x:c r="L32" t="str">
-        <x:v>success_score;performance_score;stability_score;cost_efficiency_score</x:v>
+        <x:v>success_score;performance_score;cost_efficiency_score</x:v>
       </x:c>
       <x:c r="M32" t="str">
         <x:v>weighted_score</x:v>
@@ -8636,7 +8636,7 @@
         <x:v>TBD</x:v>
       </x:c>
       <x:c r="R32" t="str">
-        <x:v>0.8.0</x:v>
+        <x:v>0.11.0</x:v>
       </x:c>
       <x:c r="S32" s="21" t="n">
         <x:v>46219</x:v>
@@ -8646,7 +8646,7 @@
         <x:v>src/model_operations.py</x:v>
       </x:c>
       <x:c r="V32" t="str">
-        <x:v>成功率、性能、稳定性和成本效率按配置融合</x:v>
+        <x:v>稳定性已包含在性能评分中，不再单独重复加权</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -9396,7 +9396,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09a266a2a19a4fd2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra62fe2bcb79e4cd7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14977,7 +14977,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R626d25ecabf1493c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd3270bd181f497c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15352,7 +15352,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5262b3b7c2d941e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf88232d781f44df5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15778,7 +15778,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f2cda8f6e264043"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6aa90a76894d49e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16070,7 +16070,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4525c26d40ea4740"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R552b6c5965b74437"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16410,7 +16410,33 @@
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="B12"/>
+      <x:c r="A12" t="str">
+        <x:v>0.11.0</x:v>
+      </x:c>
+      <x:c r="B12" s="21" t="n">
+        <x:v>46226</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>fix</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>移除模型健康指数对稳定性评分的重复加权；性能评分继续包含稳定性</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>AI Monitoring Project</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>approved</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>健康指数权重调整为成功率35%、性能50%、成本效率15%，需重建运营评分及下游输出</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="B13"/>
@@ -16684,7 +16710,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bdb237312584556"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra13aa5a220c54c70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17248,7 +17274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3611b1a57f5c49ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdddde5cee3294648"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17765,7 +17791,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8804abdb906c4c81"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re33a4369116c4dee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Expand calibrated scoring and 90-day simulations
</commit_message>
<xml_diff>
--- a/docs/ai_monitoring_metric_dictionary.xlsx
+++ b/docs/ai_monitoring_metric_dictionary.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readme" sheetId="1" r:id="R83b3e0835b2740e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrics" sheetId="2" r:id="Rd7a71123dde44659"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fields" sheetId="3" r:id="Ra62d25f34d9b48ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alert Rules" sheetId="4" r:id="R42ebbcbcce7d46ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimensions" sheetId="5" r:id="Re474d66468264821"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config Values" sheetId="6" r:id="R81566ca83c334479"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version History" sheetId="7" r:id="Re368677e26d341f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composite Rules" sheetId="8" r:id="Rb4efe5d3c1194968"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Conditions" sheetId="9" r:id="R2e0bd43fad2246c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fusion Strategies" sheetId="10" r:id="R58ac61144a89462c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fusion Grading" sheetId="11" r:id="R52c587be9846496b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Probes" sheetId="12" r:id="R05256f45d8ce4a44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Probe Assertions" sheetId="13" r:id="R45946a05cf4e4d40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Severity Policy" sheetId="14" r:id="Rda913d51cdd340e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Policy" sheetId="15" r:id="R6e6268d4fb4645a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Tasks" sheetId="16" r:id="R08c8c0c628d746d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagnosis Policy" sheetId="17" r:id="Rb6009eba43d547fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Policy" sheetId="18" r:id="Rf0db931b35c34f14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readme" sheetId="1" r:id="R9cae793e1a7a4bc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrics" sheetId="2" r:id="R35d42461d28b4e07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fields" sheetId="3" r:id="R12d6e2fb884c4072"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alert Rules" sheetId="4" r:id="Rf310c6b5210c45ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimensions" sheetId="5" r:id="R22592c9e4cb8414f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config Values" sheetId="6" r:id="R7b727289cafc4436"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version History" sheetId="7" r:id="Ra899f7a5d193408b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composite Rules" sheetId="8" r:id="R139de2271d394096"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Conditions" sheetId="9" r:id="R6597a553d25944e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fusion Strategies" sheetId="10" r:id="R2bf8eb4b01684b72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fusion Grading" sheetId="11" r:id="R1b403588fc834ada"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Probes" sheetId="12" r:id="R903e05c302264261"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Probe Assertions" sheetId="13" r:id="R75717855d02444c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Severity Policy" sheetId="14" r:id="Rde3ca84d921846cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Policy" sheetId="15" r:id="Reb81374d6f9045c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Tasks" sheetId="16" r:id="R342627c3b7c842bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagnosis Policy" sheetId="17" r:id="R882f6b99a3dc44a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Policy" sheetId="18" r:id="R89cffc740f0449ac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1700,7 +1700,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="28" t="str">
-        <x:v>Version 0.11.0 | Removed duplicate stability weighting from model health score</x:v>
+        <x:v>Version 0.12.0 | Relative self-baseline scoring for latency and cost</x:v>
       </x:c>
       <x:c r="B3" s="28"/>
       <x:c r="C3" s="28"/>
@@ -2161,7 +2161,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R144b083b98524f02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R006a99e7a1f742f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2358,7 +2358,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fa6814d83a142ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafa49d56fb004aff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2866,7 +2866,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb51ef5fe4b16479f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfedd0d2c956c4b80"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3217,7 +3217,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78b9a933238d4227"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb14caf1414814d33"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3412,7 +3412,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc7b162c88cd4168"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac622d4d12b64352"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3496,32 +3496,34 @@
         <x:v>latency</x:v>
       </x:c>
       <x:c r="D2" s="149" t="str">
-        <x:v>p50_latency_ms</x:v>
+        <x:v>p50_latency_ratio</x:v>
       </x:c>
       <x:c r="E2" s="149" t="str">
-        <x:v>lower_better</x:v>
+        <x:v>relative_lower</x:v>
       </x:c>
       <x:c r="F2" s="150" t="n">
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="G2" s="151" t="n">
-        <x:v>2000</x:v>
-      </x:c>
-      <x:c r="H2" s="151"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H2" s="151" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
       <x:c r="I2" s="150"/>
       <x:c r="J2" s="150"/>
       <x:c r="K2" s="149"/>
       <x:c r="L2" s="149" t="str">
-        <x:v>ms</x:v>
+        <x:v>ratio</x:v>
       </x:c>
       <x:c r="M2" s="149" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="N2" s="149" t="str">
-        <x:v>0.6.0</x:v>
+        <x:v>0.12.0</x:v>
       </x:c>
       <x:c r="O2" s="149" t="str">
-        <x:v>P50不高于目标得满分</x:v>
+        <x:v>P50相对模型自身前7日基线；等于基线80分</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="32" customHeight="1">
@@ -3535,32 +3537,34 @@
         <x:v>latency</x:v>
       </x:c>
       <x:c r="D3" s="149" t="str">
-        <x:v>p95_latency_ms</x:v>
+        <x:v>p95_latency_ratio</x:v>
       </x:c>
       <x:c r="E3" s="149" t="str">
-        <x:v>lower_better</x:v>
+        <x:v>relative_lower</x:v>
       </x:c>
       <x:c r="F3" s="150" t="n">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G3" s="151" t="n">
-        <x:v>3000</x:v>
-      </x:c>
-      <x:c r="H3" s="151"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H3" s="151" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
       <x:c r="I3" s="150"/>
       <x:c r="J3" s="150"/>
       <x:c r="K3" s="149"/>
       <x:c r="L3" s="149" t="str">
-        <x:v>ms</x:v>
+        <x:v>ratio</x:v>
       </x:c>
       <x:c r="M3" s="149" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="N3" s="149" t="str">
-        <x:v>0.6.0</x:v>
+        <x:v>0.12.0</x:v>
       </x:c>
       <x:c r="O3" s="149" t="str">
-        <x:v>P95作为延迟主指标</x:v>
+        <x:v>P95作为主要响应速度指标；相对自身基线评分</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
@@ -3574,32 +3578,34 @@
         <x:v>latency</x:v>
       </x:c>
       <x:c r="D4" s="149" t="str">
-        <x:v>p99_latency_ms</x:v>
+        <x:v>p99_latency_ratio</x:v>
       </x:c>
       <x:c r="E4" s="149" t="str">
-        <x:v>lower_better</x:v>
+        <x:v>relative_lower</x:v>
       </x:c>
       <x:c r="F4" s="150" t="n">
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="G4" s="151" t="n">
-        <x:v>4500</x:v>
-      </x:c>
-      <x:c r="H4" s="151"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H4" s="151" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
       <x:c r="I4" s="150"/>
       <x:c r="J4" s="150"/>
       <x:c r="K4" s="149"/>
       <x:c r="L4" s="149" t="str">
-        <x:v>ms</x:v>
+        <x:v>ratio</x:v>
       </x:c>
       <x:c r="M4" s="149" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="N4" s="149" t="str">
-        <x:v>0.6.0</x:v>
+        <x:v>0.12.0</x:v>
       </x:c>
       <x:c r="O4" s="149" t="str">
-        <x:v>P99反映尾部性能</x:v>
+        <x:v>P99反映尾部性能；相对自身基线评分</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="32" customHeight="1">
@@ -3697,7 +3703,7 @@
         <x:v>passthrough</x:v>
       </x:c>
       <x:c r="F7" s="150" t="n">
-        <x:v>0.7</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="G7" s="151"/>
       <x:c r="H7" s="151"/>
@@ -3711,10 +3717,10 @@
         <x:v>active</x:v>
       </x:c>
       <x:c r="N7" s="149" t="str">
-        <x:v>0.6.0</x:v>
+        <x:v>0.12.0</x:v>
       </x:c>
       <x:c r="O7" s="149" t="str">
-        <x:v>性能评分以延迟得分为主</x:v>
+        <x:v>性能评分以相对自身基线的响应速度为主</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="32" customHeight="1">
@@ -3734,7 +3740,7 @@
         <x:v>passthrough</x:v>
       </x:c>
       <x:c r="F8" s="150" t="n">
-        <x:v>0.3</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="G8" s="151"/>
       <x:c r="H8" s="151"/>
@@ -3748,10 +3754,10 @@
         <x:v>active</x:v>
       </x:c>
       <x:c r="N8" s="149" t="str">
-        <x:v>0.6.0</x:v>
+        <x:v>0.12.0</x:v>
       </x:c>
       <x:c r="O8" s="149" t="str">
-        <x:v>性能评分同时考虑稳定性</x:v>
+        <x:v>稳定性作为性能评分的辅助约束</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="32" customHeight="1">
@@ -3804,32 +3810,34 @@
         <x:v>cost_efficiency</x:v>
       </x:c>
       <x:c r="D10" s="149" t="str">
-        <x:v>cost_per_request</x:v>
+        <x:v>cost_per_request_ratio</x:v>
       </x:c>
       <x:c r="E10" s="149" t="str">
-        <x:v>lower_better</x:v>
+        <x:v>relative_lower</x:v>
       </x:c>
       <x:c r="F10" s="150" t="n">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G10" s="151" t="n">
-        <x:v>0.0012</x:v>
-      </x:c>
-      <x:c r="H10" s="151"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H10" s="151" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
       <x:c r="I10" s="150"/>
       <x:c r="J10" s="150"/>
       <x:c r="K10" s="149"/>
       <x:c r="L10" s="149" t="str">
-        <x:v>currency/request</x:v>
+        <x:v>ratio</x:v>
       </x:c>
       <x:c r="M10" s="149" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="N10" s="149" t="str">
-        <x:v>0.6.0</x:v>
+        <x:v>0.12.0</x:v>
       </x:c>
       <x:c r="O10" s="149" t="str">
-        <x:v>首版实验目标，可按价格版本调整</x:v>
+        <x:v>单请求成本相对模型自身前7日基线；等于基线80分</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="32" customHeight="1">
@@ -3843,32 +3851,34 @@
         <x:v>cost_efficiency</x:v>
       </x:c>
       <x:c r="D11" s="149" t="str">
-        <x:v>cost_per_1k_tokens</x:v>
+        <x:v>cost_per_1k_tokens_ratio</x:v>
       </x:c>
       <x:c r="E11" s="149" t="str">
-        <x:v>lower_better</x:v>
+        <x:v>relative_lower</x:v>
       </x:c>
       <x:c r="F11" s="150" t="n">
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="G11" s="151" t="n">
-        <x:v>0.0016</x:v>
-      </x:c>
-      <x:c r="H11" s="151"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H11" s="151" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
       <x:c r="I11" s="150"/>
       <x:c r="J11" s="150"/>
       <x:c r="K11" s="149"/>
       <x:c r="L11" s="149" t="str">
-        <x:v>currency/1k-token</x:v>
+        <x:v>ratio</x:v>
       </x:c>
       <x:c r="M11" s="149" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="N11" s="149" t="str">
-        <x:v>0.6.0</x:v>
+        <x:v>0.12.0</x:v>
       </x:c>
       <x:c r="O11" s="149" t="str">
-        <x:v>首版实验目标，可按价格版本调整</x:v>
+        <x:v>千Token成本相对模型自身前7日基线；识别价格或路由变化</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="32" customHeight="1">
@@ -3882,10 +3892,10 @@
         <x:v>cost_efficiency</x:v>
       </x:c>
       <x:c r="D12" s="149" t="str">
-        <x:v>cost_trend_ratio</x:v>
+        <x:v>tokens_per_request_ratio</x:v>
       </x:c>
       <x:c r="E12" s="149" t="str">
-        <x:v>lower_better</x:v>
+        <x:v>relative_lower</x:v>
       </x:c>
       <x:c r="F12" s="150" t="n">
         <x:v>0.2</x:v>
@@ -3893,7 +3903,9 @@
       <x:c r="G12" s="151" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H12" s="151"/>
+      <x:c r="H12" s="151" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
       <x:c r="I12" s="150"/>
       <x:c r="J12" s="150"/>
       <x:c r="K12" s="149"/>
@@ -3904,10 +3916,10 @@
         <x:v>active</x:v>
       </x:c>
       <x:c r="N12" s="149" t="str">
-        <x:v>0.6.0</x:v>
+        <x:v>0.12.0</x:v>
       </x:c>
       <x:c r="O12" s="149" t="str">
-        <x:v>当前窗口成本不高于基线得满分</x:v>
+        <x:v>单请求Token相对模型自身前7日基线；识别用量结构变化</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="32" customHeight="1">
@@ -3927,7 +3939,7 @@
         <x:v>passthrough</x:v>
       </x:c>
       <x:c r="F13" s="150" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.3</x:v>
       </x:c>
       <x:c r="G13" s="151"/>
       <x:c r="H13" s="151"/>
@@ -3941,10 +3953,10 @@
         <x:v>active</x:v>
       </x:c>
       <x:c r="N13" s="149" t="str">
-        <x:v>0.6.0</x:v>
+        <x:v>0.12.0</x:v>
       </x:c>
       <x:c r="O13" s="149" t="str">
-        <x:v>避免低价低质模型获得过高排名</x:v>
+        <x:v>质量保障占成本总评分30%，防止以低价牺牲质量</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="32" customHeight="1">
@@ -3964,7 +3976,7 @@
         <x:v>passthrough</x:v>
       </x:c>
       <x:c r="F14" s="150" t="n">
-        <x:v>0.4</x:v>
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="G14" s="151"/>
       <x:c r="H14" s="151"/>
@@ -3978,10 +3990,10 @@
         <x:v>active</x:v>
       </x:c>
       <x:c r="N14" s="149" t="str">
-        <x:v>0.6.0</x:v>
+        <x:v>0.12.0</x:v>
       </x:c>
       <x:c r="O14" s="149" t="str">
-        <x:v>成本效率占40%</x:v>
+        <x:v>成本效率占成本总评分70%，作为主要构成</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="32" customHeight="1">
@@ -5154,7 +5166,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f569c11fa2f46a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45ae698222794d1b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5480,7 +5492,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5313b656fb224b9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65ca1d48b84c4e06"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5825,7 +5837,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4e148933d234aea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd45faa5df98848a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6528,7 +6540,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd51da43ba80945d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c66f02ec7b24b47"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8006,7 +8018,7 @@
         <x:v>按配置权重融合P50、P95和P99后的0到100分</x:v>
       </x:c>
       <x:c r="F23" t="str">
-        <x:v>WEIGHTED_SCORE(p50_latency_ms,p95_latency_ms,p99_latency_ms)</x:v>
+        <x:v>WEIGHTED_SCORE(p50_latency_ratio,p95_latency_ratio,p99_latency_ratio)</x:v>
       </x:c>
       <x:c r="G23" t="str">
         <x:v>score</x:v>
@@ -8024,7 +8036,7 @@
         <x:v>model_operating_scores</x:v>
       </x:c>
       <x:c r="L23" t="str">
-        <x:v>p50_latency_ms;p95_latency_ms;p99_latency_ms</x:v>
+        <x:v>p50_latency_ratio;p95_latency_ratio;p99_latency_ratio</x:v>
       </x:c>
       <x:c r="M23" t="str">
         <x:v>weighted_score</x:v>
@@ -8052,7 +8064,7 @@
         <x:v>src/model_operations.py</x:v>
       </x:c>
       <x:c r="V23" t="str">
-        <x:v>由原始调用日志的P50/P95/P99按配置计算</x:v>
+        <x:v>相对模型自身前7日延迟基线；正常约80分</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -8138,7 +8150,7 @@
         <x:v>融合延迟得分和稳定性得分的模型性能评价</x:v>
       </x:c>
       <x:c r="F25" t="str">
-        <x:v>0.70 * latency_score + 0.30 * stability_score</x:v>
+        <x:v>0.90 * latency_score + 0.10 * stability_score</x:v>
       </x:c>
       <x:c r="G25" t="str">
         <x:v>score</x:v>
@@ -8184,7 +8196,7 @@
         <x:v>src/model_operations.py</x:v>
       </x:c>
       <x:c r="V25" t="str">
-        <x:v>由延迟得分和稳定性得分按配置计算</x:v>
+        <x:v>相对响应速度为主，稳定性作为辅助约束</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -8336,7 +8348,7 @@
         <x:v>融合单请求成本、Token单价和成本趋势的0到100分</x:v>
       </x:c>
       <x:c r="F28" t="str">
-        <x:v>WEIGHTED_SCORE(cost_per_request,cost_per_1k_tokens,cost_trend_ratio)</x:v>
+        <x:v>WEIGHTED_SCORE(cost_per_request_ratio,cost_per_1k_tokens_ratio,tokens_per_request_ratio)</x:v>
       </x:c>
       <x:c r="G28" t="str">
         <x:v>score</x:v>
@@ -8354,7 +8366,7 @@
         <x:v>model_operating_scores</x:v>
       </x:c>
       <x:c r="L28" t="str">
-        <x:v>cost_per_request;cost_per_1k_tokens;cost_trend_ratio</x:v>
+        <x:v>cost_per_request_ratio;cost_per_1k_tokens_ratio;tokens_per_request_ratio</x:v>
       </x:c>
       <x:c r="M28" t="str">
         <x:v>weighted_score</x:v>
@@ -8382,7 +8394,7 @@
         <x:v>src/model_operations.py</x:v>
       </x:c>
       <x:c r="V28" t="str">
-        <x:v>含单请求成本、Token成本和前7日趋势基线</x:v>
+        <x:v>相对模型自身前7日成本基线；正常约80分</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -8402,7 +8414,7 @@
         <x:v>综合模型质量和成本效率的性价比得分</x:v>
       </x:c>
       <x:c r="F29" t="str">
-        <x:v>0.60 * quality_score + 0.40 * cost_efficiency_score</x:v>
+        <x:v>0.30 * quality_score + 0.70 * cost_efficiency_score</x:v>
       </x:c>
       <x:c r="G29" t="str">
         <x:v>score</x:v>
@@ -8448,7 +8460,7 @@
         <x:v>src/model_operations.py</x:v>
       </x:c>
       <x:c r="V29" t="str">
-        <x:v>能力质量分与成本效率分按配置融合</x:v>
+        <x:v>成本效率为主要构成，质量作为约束</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -9396,7 +9408,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra62fe2bcb79e4cd7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3dfe5b8fb002433b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10747,10 +10759,10 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="H27" t="str">
-        <x:v>P50、P95和P99按配置权重计算的0到100分</x:v>
+        <x:v>P50、P95和P99相对模型自身基线的加权得分</x:v>
       </x:c>
       <x:c r="I27" t="str">
-        <x:v>WEIGHTED_SCORE(p50_latency_ms,p95_latency_ms,p99_latency_ms)</x:v>
+        <x:v>WEIGHTED_SCORE(p50_latency_ratio,p95_latency_ratio,p99_latency_ratio)</x:v>
       </x:c>
       <x:c r="J27" t="str">
         <x:v>internal</x:v>
@@ -10766,13 +10778,13 @@
         <x:v>TBD</x:v>
       </x:c>
       <x:c r="O27" t="str">
-        <x:v>0.8.0</x:v>
+        <x:v>0.12.0</x:v>
       </x:c>
       <x:c r="P27" s="21" t="n">
-        <x:v>46219</x:v>
+        <x:v>46231</x:v>
       </x:c>
       <x:c r="Q27" t="str">
-        <x:v>配置族latency</x:v>
+        <x:v>配置族latency；正常基线为80分</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -10849,10 +10861,10 @@
         <x:v>81</x:v>
       </x:c>
       <x:c r="H29" t="str">
-        <x:v>延迟得分与稳定性得分综合结果</x:v>
+        <x:v>相对响应速度与稳定性综合结果</x:v>
       </x:c>
       <x:c r="I29" t="str">
-        <x:v>WEIGHTED_SCORE(latency_score,stability_score)</x:v>
+        <x:v>0.90 * latency_score + 0.10 * stability_score</x:v>
       </x:c>
       <x:c r="J29" t="str">
         <x:v>internal</x:v>
@@ -10868,10 +10880,10 @@
         <x:v>TBD</x:v>
       </x:c>
       <x:c r="O29" t="str">
-        <x:v>0.8.0</x:v>
+        <x:v>0.12.0</x:v>
       </x:c>
       <x:c r="P29" s="21" t="n">
-        <x:v>46219</x:v>
+        <x:v>46231</x:v>
       </x:c>
       <x:c r="Q29" t="str">
         <x:v>配置族performance</x:v>
@@ -11002,10 +11014,10 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="H32" t="str">
-        <x:v>成本类指标按配置加权得到的0到100分</x:v>
+        <x:v>相对自身基线的成本效率得分</x:v>
       </x:c>
       <x:c r="I32" t="str">
-        <x:v>WEIGHTED_SCORE(cost_per_request,cost_per_1k_tokens,cost_trend_ratio)</x:v>
+        <x:v>WEIGHTED_SCORE(cost_per_request_ratio,cost_per_1k_tokens_ratio,tokens_per_request_ratio)</x:v>
       </x:c>
       <x:c r="J32" t="str">
         <x:v>confidential</x:v>
@@ -11021,13 +11033,13 @@
         <x:v>TBD</x:v>
       </x:c>
       <x:c r="O32" t="str">
-        <x:v>0.8.0</x:v>
+        <x:v>0.12.0</x:v>
       </x:c>
       <x:c r="P32" s="21" t="n">
-        <x:v>46219</x:v>
+        <x:v>46231</x:v>
       </x:c>
       <x:c r="Q32" t="str">
-        <x:v>配置族cost_efficiency</x:v>
+        <x:v>配置族cost_efficiency；正常基线为80分</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -11104,10 +11116,10 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="H34" t="str">
-        <x:v>质量与成本效率综合得分</x:v>
+        <x:v>成本效率为主、质量保障为约束的综合得分</x:v>
       </x:c>
       <x:c r="I34" t="str">
-        <x:v>WEIGHTED_SCORE(quality_score,cost_efficiency_score)</x:v>
+        <x:v>0.30 * quality_score + 0.70 * cost_efficiency_score</x:v>
       </x:c>
       <x:c r="J34" t="str">
         <x:v>confidential</x:v>
@@ -11123,10 +11135,10 @@
         <x:v>TBD</x:v>
       </x:c>
       <x:c r="O34" t="str">
-        <x:v>0.8.0</x:v>
+        <x:v>0.12.0</x:v>
       </x:c>
       <x:c r="P34" s="21" t="n">
-        <x:v>46219</x:v>
+        <x:v>46231</x:v>
       </x:c>
       <x:c r="Q34" t="str">
         <x:v>配置族cost_performance</x:v>
@@ -14977,7 +14989,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd3270bd181f497c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd56c29b8d44c42c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15352,7 +15364,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf88232d781f44df5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4a9642475254f38"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15778,7 +15790,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6aa90a76894d49e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4eacaadd7604044"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16070,7 +16082,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R552b6c5965b74437"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd36e8bfcc08a4b73"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16439,7 +16451,33 @@
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="B13"/>
+      <x:c r="A13" t="str">
+        <x:v>0.12.0</x:v>
+      </x:c>
+      <x:c r="B13" t="n">
+        <x:v>46231</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>feature</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>响应速度和成本效率改为相对模型自身基线评分；成本效率成为成本总评分主要构成</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>AI Monitoring Project</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>approved</x:v>
+      </x:c>
+      <x:c r="I13" t="str">
+        <x:v>需重建运营评分及下游画像、风险和诊断输出</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="B14"/>
@@ -16710,7 +16748,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra13aa5a220c54c70"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f4eddd948e64593"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17274,7 +17312,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdddde5cee3294648"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4dc2e8522e8541a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17791,7 +17829,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re33a4369116c4dee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff25c6b71bc14c6c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refine capacity diagnostics and operating data
</commit_message>
<xml_diff>
--- a/docs/ai_monitoring_metric_dictionary.xlsx
+++ b/docs/ai_monitoring_metric_dictionary.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readme" sheetId="1" r:id="R9cae793e1a7a4bc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrics" sheetId="2" r:id="R35d42461d28b4e07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fields" sheetId="3" r:id="R12d6e2fb884c4072"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alert Rules" sheetId="4" r:id="Rf310c6b5210c45ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimensions" sheetId="5" r:id="R22592c9e4cb8414f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config Values" sheetId="6" r:id="R7b727289cafc4436"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version History" sheetId="7" r:id="Ra899f7a5d193408b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composite Rules" sheetId="8" r:id="R139de2271d394096"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Conditions" sheetId="9" r:id="R6597a553d25944e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fusion Strategies" sheetId="10" r:id="R2bf8eb4b01684b72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fusion Grading" sheetId="11" r:id="R1b403588fc834ada"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Probes" sheetId="12" r:id="R903e05c302264261"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Probe Assertions" sheetId="13" r:id="R75717855d02444c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Severity Policy" sheetId="14" r:id="Rde3ca84d921846cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Policy" sheetId="15" r:id="Reb81374d6f9045c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Tasks" sheetId="16" r:id="R342627c3b7c842bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagnosis Policy" sheetId="17" r:id="R882f6b99a3dc44a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Policy" sheetId="18" r:id="R89cffc740f0449ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readme" sheetId="1" r:id="R38de8e329b3d4068"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrics" sheetId="2" r:id="Rd51d8b6ac0a44c92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fields" sheetId="3" r:id="R7e57d8253c81448c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alert Rules" sheetId="4" r:id="Rf5e6c41998eb4903"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimensions" sheetId="5" r:id="Redbf629068bb46f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config Values" sheetId="6" r:id="R8f5bdef8ed354659"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version History" sheetId="7" r:id="R876c35aa104446db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composite Rules" sheetId="8" r:id="R4c643c9786c6425e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Conditions" sheetId="9" r:id="Rc8afb19b2d004f11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fusion Strategies" sheetId="10" r:id="R7afd483be0c144e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fusion Grading" sheetId="11" r:id="R9656c3358e914f6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Probes" sheetId="12" r:id="Reffb78eff1034996"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Probe Assertions" sheetId="13" r:id="R608f175ea52849b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Severity Policy" sheetId="14" r:id="Rcbbe4d70d4b84fe9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Policy" sheetId="15" r:id="R81449268df854530"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Tasks" sheetId="16" r:id="Rb9c8662018cd4cb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagnosis Policy" sheetId="17" r:id="Re884bd71f8494820"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Policy" sheetId="18" r:id="R27b2b0c4c9274570"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1700,7 +1700,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="28" t="str">
-        <x:v>Version 0.12.0 | Relative self-baseline scoring for latency and cost</x:v>
+        <x:v>Version 0.13.0 | Sample-size-aware stability aggregation</x:v>
       </x:c>
       <x:c r="B3" s="28"/>
       <x:c r="C3" s="28"/>
@@ -2161,7 +2161,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R006a99e7a1f742f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9b4b51b929e43d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2358,7 +2358,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafa49d56fb004aff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ff41823a5464ddb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2866,7 +2866,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfedd0d2c956c4b80"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf90b648c45b4e30"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3217,7 +3217,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb14caf1414814d33"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb103391966c49df"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3412,7 +3412,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac622d4d12b64352"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e811f558b2f498e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5166,7 +5166,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45ae698222794d1b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2141470c453b4e0f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5492,7 +5492,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65ca1d48b84c4e06"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c2155265b604406"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5837,7 +5837,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd45faa5df98848a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5016ea3855e5462d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6540,7 +6540,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c66f02ec7b24b47"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d0d6429940147c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7949,10 +7949,10 @@
         <x:v>model</x:v>
       </x:c>
       <x:c r="E22" t="str">
-        <x:v>观察窗口内小时P95时延标准差与均值之比</x:v>
+        <x:v>按日调用量自适应1/3/6小时桶的P95延迟标准差与均值之比</x:v>
       </x:c>
       <x:c r="F22" t="str">
-        <x:v>STDDEV(hourly p95_latency_ms) / AVG(hourly p95_latency_ms)</x:v>
+        <x:v>STDDEV(adaptive_bucket p95_latency_ms) / AVG(adaptive_bucket p95_latency_ms)</x:v>
       </x:c>
       <x:c r="G22" t="str">
         <x:v>ratio</x:v>
@@ -7998,7 +7998,7 @@
         <x:v>src/model_operations.py</x:v>
       </x:c>
       <x:c r="V22" t="str">
-        <x:v>日内小时P95变异系数</x:v>
+        <x:v>日调用量不少于240使用1小时桶，不少于80使用3小时桶，其余使用6小时桶</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -8081,7 +8081,7 @@
         <x:v>model</x:v>
       </x:c>
       <x:c r="E24" t="str">
-        <x:v>综合延迟波动和成功率波动的0到100分</x:v>
+        <x:v>基于自适应时间桶综合延迟波动和成功率波动的0到100分</x:v>
       </x:c>
       <x:c r="F24" t="str">
         <x:v>WEIGHTED_SCORE(latency_cv,success_rate_std_pct)</x:v>
@@ -8130,7 +8130,7 @@
         <x:v>src/model_operations.py</x:v>
       </x:c>
       <x:c r="V24" t="str">
-        <x:v>由延迟波动和成功率波动按配置计算</x:v>
+        <x:v>低流量模型先扩大统计窗口，避免单次请求放大小时波动</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -9408,7 +9408,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3dfe5b8fb002433b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b2d1eb0f74b466b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10606,10 +10606,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="H24" t="str">
-        <x:v>观察窗口内小时P95时延的标准差与均值之比</x:v>
+        <x:v>按日调用量选择1/3/6小时桶后，桶级P95延迟的标准差与均值之比</x:v>
       </x:c>
       <x:c r="I24" t="str">
-        <x:v>STDDEV(p95_latency_ms) / AVG(p95_latency_ms)</x:v>
+        <x:v>STDDEV(adaptive_bucket p95_latency_ms) / AVG(adaptive_bucket p95_latency_ms)</x:v>
       </x:c>
       <x:c r="J24" t="str">
         <x:v>internal</x:v>
@@ -10625,13 +10625,13 @@
         <x:v>TBD</x:v>
       </x:c>
       <x:c r="O24" t="str">
-        <x:v>0.8.0</x:v>
+        <x:v>0.13.0</x:v>
       </x:c>
       <x:c r="P24" s="21" t="n">
-        <x:v>46219</x:v>
+        <x:v>46232</x:v>
       </x:c>
       <x:c r="Q24" t="str">
-        <x:v>无量纲；均值为0时为空</x:v>
+        <x:v>低样本模型使用自适应时间桶</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -10657,10 +10657,10 @@
         <x:v>2.5</x:v>
       </x:c>
       <x:c r="H25" t="str">
-        <x:v>观察窗口内小时成功率的标准差</x:v>
+        <x:v>按日调用量选择1/3/6小时桶后，桶级成功率的标准差</x:v>
       </x:c>
       <x:c r="I25" t="str">
-        <x:v>STDDEV(hourly success_rate)</x:v>
+        <x:v>STDDEV(adaptive_bucket success_rate)</x:v>
       </x:c>
       <x:c r="J25" t="str">
         <x:v>internal</x:v>
@@ -10676,13 +10676,13 @@
         <x:v>TBD</x:v>
       </x:c>
       <x:c r="O25" t="str">
-        <x:v>0.8.0</x:v>
+        <x:v>0.13.0</x:v>
       </x:c>
       <x:c r="P25" s="21" t="n">
-        <x:v>46219</x:v>
+        <x:v>46232</x:v>
       </x:c>
       <x:c r="Q25" t="str">
-        <x:v>单位为百分点</x:v>
+        <x:v>低样本模型使用自适应时间桶</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -14967,6 +14967,108 @@
       </x:c>
       <x:c r="Q109" t="str">
         <x:v>供看板直接展示</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" t="str">
+        <x:v>FLD-109</x:v>
+      </x:c>
+      <x:c r="B110" t="str">
+        <x:v>stability_bucket_hours</x:v>
+      </x:c>
+      <x:c r="C110" t="str">
+        <x:v>稳定性统计桶时长</x:v>
+      </x:c>
+      <x:c r="D110" t="str">
+        <x:v>derived</x:v>
+      </x:c>
+      <x:c r="E110" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="F110" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G110" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H110" t="str">
+        <x:v>按日调用量选择的稳定性统计时间桶小时数</x:v>
+      </x:c>
+      <x:c r="I110" t="str">
+        <x:v>1h if requests&gt;=240; 3h if requests&gt;=80; else 6h</x:v>
+      </x:c>
+      <x:c r="J110" t="str">
+        <x:v>internal</x:v>
+      </x:c>
+      <x:c r="K110"/>
+      <x:c r="L110" t="str">
+        <x:v>analytics_layer</x:v>
+      </x:c>
+      <x:c r="M110" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="N110" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="O110" t="str">
+        <x:v>0.13.0</x:v>
+      </x:c>
+      <x:c r="P110" t="n">
+        <x:v>46232</x:v>
+      </x:c>
+      <x:c r="Q110" t="str">
+        <x:v>降低低样本小时指标的随机波动</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" t="str">
+        <x:v>FLD-110</x:v>
+      </x:c>
+      <x:c r="B111" t="str">
+        <x:v>stability_bucket_count</x:v>
+      </x:c>
+      <x:c r="C111" t="str">
+        <x:v>稳定性有效桶数</x:v>
+      </x:c>
+      <x:c r="D111" t="str">
+        <x:v>derived</x:v>
+      </x:c>
+      <x:c r="E111" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="F111" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G111" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H111" t="str">
+        <x:v>当天实际参与稳定性计算的时间桶数量</x:v>
+      </x:c>
+      <x:c r="I111" t="str">
+        <x:v>count distinct stability_bucket</x:v>
+      </x:c>
+      <x:c r="J111" t="str">
+        <x:v>internal</x:v>
+      </x:c>
+      <x:c r="K111"/>
+      <x:c r="L111" t="str">
+        <x:v>analytics_layer</x:v>
+      </x:c>
+      <x:c r="M111" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="N111" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="O111" t="str">
+        <x:v>0.13.0</x:v>
+      </x:c>
+      <x:c r="P111" t="n">
+        <x:v>46232</x:v>
+      </x:c>
+      <x:c r="Q111" t="str">
+        <x:v>少于2个桶时稳定性不评分</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14989,7 +15091,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd56c29b8d44c42c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe6e0555a5184966"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15364,7 +15466,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4a9642475254f38"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc38f0d6e5d344df0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15790,7 +15892,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4eacaadd7604044"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d85fb040fcc4485"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16082,7 +16184,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd36e8bfcc08a4b73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R126b033277b44820"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16480,7 +16582,33 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="B14"/>
+      <x:c r="A14" t="str">
+        <x:v>0.13.0</x:v>
+      </x:c>
+      <x:c r="B14" t="n">
+        <x:v>46232</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>fix</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>稳定性改用按日调用量自适应的1/3/6小时统计桶，降低低流量模型的小样本偏差</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>AI Monitoring Project</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>approved</x:v>
+      </x:c>
+      <x:c r="I14" t="str">
+        <x:v>需重建运营评分及下游画像、风险和诊断输出</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="B15"/>
@@ -16748,7 +16876,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f4eddd948e64593"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cd695ca8a2e4fbb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17312,7 +17440,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4dc2e8522e8541a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5843791a6e4141ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17829,7 +17957,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff25c6b71bc14c6c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc49d9b46388b4813"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>